<commit_message>
initial commit mandatory XP - week2 day 3
</commit_message>
<xml_diff>
--- a/Course_plan.xlsx
+++ b/Course_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ned17\DIMA\DevelopersInstitute\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6179C1B2-C965-403A-8497-5A78DB23134F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2F320D5-F7D2-4A3C-99A9-47C227800364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{02B2EA89-8E4F-4CED-A858-D02A5E025590}"/>
+    <workbookView xWindow="-28920" yWindow="-2970" windowWidth="29040" windowHeight="15840" xr2:uid="{02B2EA89-8E4F-4CED-A858-D02A5E025590}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
   <si>
     <t>Week</t>
   </si>
@@ -81,12 +81,6 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>Evening - Lecture - Daniil Chernov, Head of Analytics, Office of CPTO at monday.com; Hackathon #1</t>
-  </si>
-  <si>
-    <t>Hackathon #2 Gen AI</t>
-  </si>
-  <si>
     <t>Ziv (/Tobi)</t>
   </si>
   <si>
@@ -100,13 +94,46 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Topics</t>
+  </si>
+  <si>
+    <t>DA overview, Preprocessing &amp; Transformation, Scipy and Basic Statistics, Data Visualization</t>
+  </si>
+  <si>
+    <t>Numpy, Intro to ML</t>
+  </si>
+  <si>
+    <t>Supervised ML, Statistics for ML</t>
+  </si>
+  <si>
+    <t>Intro to Deep Learning, Training Deep Neural Networks, Convolutional Neural Networks, Recurrent Neural Networks</t>
+  </si>
+  <si>
+    <t>the Rise of LLMs, Deep Dive into Advanced Transformer and LLM concept, BERT, Fine tuning of LLMs</t>
+  </si>
+  <si>
+    <t>NLP - preprocessing; Vector DBs and RAG chatbots; RAG; Evaluation, Benchmarking/Integration</t>
+  </si>
+  <si>
+    <t>Hackathon #2 Gen AI (Group Project)</t>
+  </si>
+  <si>
+    <t>MCP, Agentic AI - from setup to frameworks; MCP+Agentic AI solutions</t>
+  </si>
+  <si>
+    <t>Basic Prompting, Documents w Claude, Cross Referenced Analysis, Claude Cowork Delegating Task</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evening - Lecture - Daniil Chernov, Head of Analytics, Office of CPTO at monday.com; Hackathon #1 (Group Project) - </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -114,13 +141,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF66"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -135,15 +182,58 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFFF66"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -452,227 +542,274 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{94232BE0-A001-4A15-B061-649826CD6E04}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="52.5703125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="64.85546875" style="5" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" s="12" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="F1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="7">
         <v>46313</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+    </row>
+    <row r="3" spans="1:6" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="10">
         <f>B2+7</f>
         <v>46320</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="9" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="E3" s="11"/>
+      <c r="F3" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="13" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="4">
         <f>B3+7+1</f>
         <v>46328</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="E4" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="4">
         <f t="shared" ref="B4:B13" si="0">B4+7</f>
         <v>46335</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="E5" s="5"/>
+      <c r="F5" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="4">
         <f t="shared" si="0"/>
         <v>46342</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="E6" s="5"/>
+      <c r="F6" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="3">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="4">
         <f t="shared" si="0"/>
         <v>46349</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="3" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="E7" s="5"/>
+      <c r="F7" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="4">
         <f t="shared" si="0"/>
         <v>46356</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="E8" s="5"/>
+      <c r="F8" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="3">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="4">
         <f t="shared" si="0"/>
         <v>46363</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="3" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="E9" s="5"/>
+      <c r="F9" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="3">
         <v>9</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="4">
         <f t="shared" si="0"/>
         <v>46370</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D10" t="s">
-        <v>20</v>
-      </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="D10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="5"/>
+    </row>
+    <row r="11" spans="1:6" s="13" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="3">
         <v>10</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="4">
         <f t="shared" si="0"/>
         <v>46377</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="D11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="3">
         <v>11</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="4">
         <f t="shared" si="0"/>
         <v>46384</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="D12" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="3">
         <v>12</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="4">
         <f t="shared" si="0"/>
         <v>46391</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D13" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B14" s="1">
+      <c r="D13" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+    </row>
+    <row r="14" spans="1:6" s="13" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="3"/>
+      <c r="B14" s="4">
         <v>46397</v>
       </c>
-      <c r="C14" t="s">
-        <v>23</v>
-      </c>
+      <c r="C14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="3"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>